<commit_message>
Raise Lot A production pricing to 185K and mark payment terms as preferred
Lot A arrangements now total 510,000 (325,000 hotel package at cost +
185,000 production & services), with increases weighted toward AV and
production items. Payment terms reworded as preferred/negotiable, with
the 50% advance tied to the mandatory hotel advance payment.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TF4abcCWc11H47Q8mehd7k
</commit_message>
<xml_diff>
--- a/leap2026/PSEB_LEAP2026_Commercial_Proposal_Miradore.xlsx
+++ b/leap2026/PSEB_LEAP2026_Commercial_Proposal_Miradore.xlsx
@@ -180,7 +180,7 @@
     <t xml:space="preserve">PAYMENT TERMS &amp; KEY CONDITIONS</t>
   </si>
   <si>
-    <t xml:space="preserve">•  Payment Terms: 50% advance upon confirmation / work order; 30% two (2) days before the event; 20% balance after the event, upon successful delivery and verification.</t>
+    <t xml:space="preserve">•  Preferred Payment Terms (negotiable): 50% advance upon confirmation / work order — primarily to cover the mandatory advance payment required by Crowne Plaza Riyadh RDC to secure the venue, plus mobilization of fabrication and long-lead items; 30% two (2) days before the event; 20% balance after the event, upon successful delivery and verification.</t>
   </si>
   <si>
     <t xml:space="preserve">•  The Crowne Plaza Riyadh RDC venue &amp; catering package (Lot A, item A.1) is passed through at actual hotel package cost, with no markup.</t>
@@ -1992,11 +1992,11 @@
       </c>
       <c r="C13" s="25" t="n">
         <f aca="false">'Lot A - Forum'!F20</f>
-        <v>468350</v>
+        <v>510000</v>
       </c>
       <c r="D13" s="25" t="n">
         <f aca="false">ROUND(C13*Summary!$C$9,0)</f>
-        <v>35360425</v>
+        <v>38505000</v>
       </c>
       <c r="E13" s="26" t="s">
         <v>30</v>
@@ -2024,11 +2024,11 @@
       </c>
       <c r="C15" s="28" t="n">
         <f aca="false">C13+C14</f>
-        <v>786030</v>
+        <v>827680</v>
       </c>
       <c r="D15" s="28" t="n">
         <f aca="false">ROUND(C15*Summary!$C$9,0)</f>
-        <v>59345265</v>
+        <v>62489840</v>
       </c>
       <c r="E15" s="29"/>
     </row>
@@ -2038,11 +2038,11 @@
       </c>
       <c r="C16" s="25" t="n">
         <f aca="false">'Lot A - Forum'!F21+'Lot B - Pavilion'!F12</f>
-        <v>94323.6</v>
+        <v>99321.6</v>
       </c>
       <c r="D16" s="25" t="n">
         <f aca="false">ROUND(C16*Summary!$C$9,0)</f>
-        <v>7121432</v>
+        <v>7498781</v>
       </c>
       <c r="E16" s="26" t="s">
         <v>34</v>
@@ -2054,11 +2054,11 @@
       </c>
       <c r="C17" s="28" t="n">
         <f aca="false">C15+C16</f>
-        <v>880353.6</v>
+        <v>927001.6</v>
       </c>
       <c r="D17" s="28" t="n">
         <f aca="false">ROUND(C17*Summary!$C$9,0)</f>
-        <v>66466697</v>
+        <v>69988621</v>
       </c>
       <c r="E17" s="29"/>
     </row>
@@ -2068,11 +2068,11 @@
       </c>
       <c r="C18" s="25" t="n">
         <f aca="false">ROUND(C17*Summary!$C$7,2)</f>
-        <v>132053.04</v>
+        <v>139050.24</v>
       </c>
       <c r="D18" s="25" t="n">
         <f aca="false">ROUND(C18*Summary!$C$9,0)</f>
-        <v>9970005</v>
+        <v>10498293</v>
       </c>
       <c r="E18" s="26"/>
     </row>
@@ -2082,11 +2082,11 @@
       </c>
       <c r="C19" s="31" t="n">
         <f aca="false">C17+C18</f>
-        <v>1012406.64</v>
+        <v>1066051.84</v>
       </c>
       <c r="D19" s="32" t="n">
         <f aca="false">ROUND(C19*Summary!$C$9,0)</f>
-        <v>76436701</v>
+        <v>80486914</v>
       </c>
       <c r="E19" s="33" t="s">
         <v>38</v>
@@ -2120,15 +2120,15 @@
       </c>
       <c r="C23" s="34" t="n">
         <f aca="false">'Lot A - Forum'!F22</f>
-        <v>524552</v>
+        <v>571200</v>
       </c>
       <c r="D23" s="34" t="n">
         <f aca="false">'Lot A - Forum'!F24</f>
-        <v>603234.8</v>
+        <v>656880</v>
       </c>
       <c r="E23" s="25" t="n">
         <f aca="false">ROUND(D23*Summary!$C$9,0)</f>
-        <v>45544227</v>
+        <v>49594440</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2156,7 +2156,7 @@
       <c r="D26" s="21"/>
       <c r="E26" s="21"/>
     </row>
-    <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="35" t="s">
         <v>47</v>
       </c>
@@ -2370,19 +2370,19 @@
         <v>71</v>
       </c>
       <c r="E6" s="46" t="n">
-        <v>13000</v>
+        <v>18500</v>
       </c>
       <c r="F6" s="47" t="n">
         <f aca="false">ROUND(C6*E6,2)</f>
-        <v>13000</v>
+        <v>18500</v>
       </c>
       <c r="G6" s="48" t="n">
         <f aca="false">ROUND(E6*Summary!$C$9,0)</f>
-        <v>981500</v>
+        <v>1396750</v>
       </c>
       <c r="H6" s="48" t="n">
         <f aca="false">ROUND(F6*Summary!$C$9,0)</f>
-        <v>981500</v>
+        <v>1396750</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2399,19 +2399,19 @@
         <v>71</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>9500</v>
+        <v>12500</v>
       </c>
       <c r="F7" s="41" t="n">
         <f aca="false">ROUND(C7*E7,2)</f>
-        <v>9500</v>
+        <v>12500</v>
       </c>
       <c r="G7" s="42" t="n">
         <f aca="false">ROUND(E7*Summary!$C$9,0)</f>
-        <v>717250</v>
+        <v>943750</v>
       </c>
       <c r="H7" s="42" t="n">
         <f aca="false">ROUND(F7*Summary!$C$9,0)</f>
-        <v>717250</v>
+        <v>943750</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2428,19 +2428,19 @@
         <v>40</v>
       </c>
       <c r="E8" s="46" t="n">
-        <v>15750</v>
+        <v>19500</v>
       </c>
       <c r="F8" s="47" t="n">
         <f aca="false">ROUND(C8*E8,2)</f>
-        <v>15750</v>
+        <v>19500</v>
       </c>
       <c r="G8" s="48" t="n">
         <f aca="false">ROUND(E8*Summary!$C$9,0)</f>
-        <v>1189125</v>
+        <v>1472250</v>
       </c>
       <c r="H8" s="48" t="n">
         <f aca="false">ROUND(F8*Summary!$C$9,0)</f>
-        <v>1189125</v>
+        <v>1472250</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2457,19 +2457,19 @@
         <v>71</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>8400</v>
+        <v>10500</v>
       </c>
       <c r="F9" s="41" t="n">
         <f aca="false">ROUND(C9*E9,2)</f>
-        <v>8400</v>
+        <v>10500</v>
       </c>
       <c r="G9" s="42" t="n">
         <f aca="false">ROUND(E9*Summary!$C$9,0)</f>
-        <v>634200</v>
+        <v>792750</v>
       </c>
       <c r="H9" s="42" t="n">
         <f aca="false">ROUND(F9*Summary!$C$9,0)</f>
-        <v>634200</v>
+        <v>792750</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2486,19 +2486,19 @@
         <v>71</v>
       </c>
       <c r="E10" s="46" t="n">
-        <v>10800</v>
+        <v>13500</v>
       </c>
       <c r="F10" s="47" t="n">
         <f aca="false">ROUND(C10*E10,2)</f>
-        <v>10800</v>
+        <v>13500</v>
       </c>
       <c r="G10" s="48" t="n">
         <f aca="false">ROUND(E10*Summary!$C$9,0)</f>
-        <v>815400</v>
+        <v>1019250</v>
       </c>
       <c r="H10" s="48" t="n">
         <f aca="false">ROUND(F10*Summary!$C$9,0)</f>
-        <v>815400</v>
+        <v>1019250</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2515,19 +2515,19 @@
         <v>82</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>1025</v>
+        <v>1350</v>
       </c>
       <c r="F11" s="41" t="n">
         <f aca="false">ROUND(C11*E11,2)</f>
-        <v>4100</v>
+        <v>5400</v>
       </c>
       <c r="G11" s="42" t="n">
         <f aca="false">ROUND(E11*Summary!$C$9,0)</f>
-        <v>77388</v>
+        <v>101925</v>
       </c>
       <c r="H11" s="42" t="n">
         <f aca="false">ROUND(F11*Summary!$C$9,0)</f>
-        <v>309550</v>
+        <v>407700</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2544,19 +2544,19 @@
         <v>71</v>
       </c>
       <c r="E12" s="46" t="n">
-        <v>19900</v>
+        <v>26500</v>
       </c>
       <c r="F12" s="47" t="n">
         <f aca="false">ROUND(C12*E12,2)</f>
-        <v>19900</v>
+        <v>26500</v>
       </c>
       <c r="G12" s="48" t="n">
         <f aca="false">ROUND(E12*Summary!$C$9,0)</f>
-        <v>1502450</v>
+        <v>2000750</v>
       </c>
       <c r="H12" s="48" t="n">
         <f aca="false">ROUND(F12*Summary!$C$9,0)</f>
-        <v>1502450</v>
+        <v>2000750</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2573,19 +2573,19 @@
         <v>71</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>26500</v>
+        <v>34500</v>
       </c>
       <c r="F13" s="41" t="n">
         <f aca="false">ROUND(C13*E13,2)</f>
-        <v>26500</v>
+        <v>34500</v>
       </c>
       <c r="G13" s="42" t="n">
         <f aca="false">ROUND(E13*Summary!$C$9,0)</f>
-        <v>2000750</v>
+        <v>2604750</v>
       </c>
       <c r="H13" s="42" t="n">
         <f aca="false">ROUND(F13*Summary!$C$9,0)</f>
-        <v>2000750</v>
+        <v>2604750</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2602,19 +2602,19 @@
         <v>82</v>
       </c>
       <c r="E14" s="46" t="n">
-        <v>2400</v>
+        <v>3150</v>
       </c>
       <c r="F14" s="47" t="n">
         <f aca="false">ROUND(C14*E14,2)</f>
-        <v>9600</v>
+        <v>12600</v>
       </c>
       <c r="G14" s="48" t="n">
         <f aca="false">ROUND(E14*Summary!$C$9,0)</f>
-        <v>181200</v>
+        <v>237825</v>
       </c>
       <c r="H14" s="48" t="n">
         <f aca="false">ROUND(F14*Summary!$C$9,0)</f>
-        <v>724800</v>
+        <v>951300</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2631,19 +2631,19 @@
         <v>71</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>4500</v>
+        <v>5000</v>
       </c>
       <c r="F15" s="41" t="n">
         <f aca="false">ROUND(C15*E15,2)</f>
-        <v>4500</v>
+        <v>5000</v>
       </c>
       <c r="G15" s="42" t="n">
         <f aca="false">ROUND(E15*Summary!$C$9,0)</f>
-        <v>339750</v>
+        <v>377500</v>
       </c>
       <c r="H15" s="42" t="n">
         <f aca="false">ROUND(F15*Summary!$C$9,0)</f>
-        <v>339750</v>
+        <v>377500</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2684,19 +2684,19 @@
         <v>71</v>
       </c>
       <c r="E17" s="40" t="n">
-        <v>4500</v>
+        <v>5500</v>
       </c>
       <c r="F17" s="41" t="n">
         <f aca="false">ROUND(C17*E17,2)</f>
-        <v>4500</v>
+        <v>5500</v>
       </c>
       <c r="G17" s="42" t="n">
         <f aca="false">ROUND(E17*Summary!$C$9,0)</f>
-        <v>339750</v>
+        <v>415250</v>
       </c>
       <c r="H17" s="42" t="n">
         <f aca="false">ROUND(F17*Summary!$C$9,0)</f>
-        <v>339750</v>
+        <v>415250</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2713,19 +2713,19 @@
         <v>71</v>
       </c>
       <c r="E18" s="46" t="n">
-        <v>8500</v>
+        <v>11500</v>
       </c>
       <c r="F18" s="47" t="n">
         <f aca="false">ROUND(C18*E18,2)</f>
-        <v>8500</v>
+        <v>11500</v>
       </c>
       <c r="G18" s="48" t="n">
         <f aca="false">ROUND(E18*Summary!$C$9,0)</f>
-        <v>641750</v>
+        <v>868250</v>
       </c>
       <c r="H18" s="48" t="n">
         <f aca="false">ROUND(F18*Summary!$C$9,0)</f>
-        <v>641750</v>
+        <v>868250</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2742,19 +2742,19 @@
         <v>101</v>
       </c>
       <c r="E19" s="40" t="n">
-        <v>830</v>
+        <v>950</v>
       </c>
       <c r="F19" s="41" t="n">
         <f aca="false">ROUND(C19*E19,2)</f>
-        <v>8300</v>
+        <v>9500</v>
       </c>
       <c r="G19" s="42" t="n">
         <f aca="false">ROUND(E19*Summary!$C$9,0)</f>
-        <v>62665</v>
+        <v>71725</v>
       </c>
       <c r="H19" s="42" t="n">
         <f aca="false">ROUND(F19*Summary!$C$9,0)</f>
-        <v>626650</v>
+        <v>717250</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2767,12 +2767,12 @@
       <c r="E20" s="52"/>
       <c r="F20" s="53" t="n">
         <f aca="false">SUM(F5:F19)</f>
-        <v>468350</v>
+        <v>510000</v>
       </c>
       <c r="G20" s="54"/>
       <c r="H20" s="55" t="n">
         <f aca="false">ROUND(F20*Summary!$C$9,0)</f>
-        <v>35360425</v>
+        <v>38505000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2785,12 +2785,12 @@
       <c r="E21" s="56"/>
       <c r="F21" s="57" t="n">
         <f aca="false">ROUND(F20*Summary!$C$8,2)</f>
-        <v>56202</v>
+        <v>61200</v>
       </c>
       <c r="G21" s="58"/>
       <c r="H21" s="42" t="n">
         <f aca="false">ROUND(F21*Summary!$C$9,0)</f>
-        <v>4243251</v>
+        <v>4620600</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2803,12 +2803,12 @@
       <c r="E22" s="52"/>
       <c r="F22" s="53" t="n">
         <f aca="false">F20+F21</f>
-        <v>524552</v>
+        <v>571200</v>
       </c>
       <c r="G22" s="54"/>
       <c r="H22" s="55" t="n">
         <f aca="false">ROUND(F22*Summary!$C$9,0)</f>
-        <v>39603676</v>
+        <v>43125600</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2821,12 +2821,12 @@
       <c r="E23" s="56"/>
       <c r="F23" s="57" t="n">
         <f aca="false">ROUND(F22*Summary!$C$7,2)</f>
-        <v>78682.8</v>
+        <v>85680</v>
       </c>
       <c r="G23" s="58"/>
       <c r="H23" s="42" t="n">
         <f aca="false">ROUND(F23*Summary!$C$9,0)</f>
-        <v>5940551</v>
+        <v>6468840</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2839,12 +2839,12 @@
       <c r="E24" s="59"/>
       <c r="F24" s="31" t="n">
         <f aca="false">F22+F23</f>
-        <v>603234.8</v>
+        <v>656880</v>
       </c>
       <c r="G24" s="60"/>
       <c r="H24" s="61" t="n">
         <f aca="false">ROUND(F24*Summary!$C$9,0)</f>
-        <v>45544227</v>
+        <v>49594440</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3574,18 +3574,18 @@
       </c>
       <c r="C6" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F6</f>
-        <v>13000</v>
+        <v>18500</v>
       </c>
       <c r="D6" s="72" t="n">
         <v>10000</v>
       </c>
       <c r="E6" s="71" t="n">
         <f aca="false">C6-D6</f>
-        <v>3000</v>
+        <v>8500</v>
       </c>
       <c r="F6" s="73" t="n">
         <f aca="false">IF(D6=0,"n/a",C6/D6-1)</f>
-        <v>0.3</v>
+        <v>0.85</v>
       </c>
       <c r="G6" s="26" t="s">
         <v>178</v>
@@ -3600,18 +3600,18 @@
       </c>
       <c r="C7" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F7</f>
-        <v>9500</v>
+        <v>12500</v>
       </c>
       <c r="D7" s="72" t="n">
         <v>7400</v>
       </c>
       <c r="E7" s="71" t="n">
         <f aca="false">C7-D7</f>
-        <v>2100</v>
+        <v>5100</v>
       </c>
       <c r="F7" s="73" t="n">
         <f aca="false">IF(D7=0,"n/a",C7/D7-1)</f>
-        <v>0.283783783783784</v>
+        <v>0.689189189189189</v>
       </c>
       <c r="G7" s="26" t="s">
         <v>180</v>
@@ -3626,18 +3626,18 @@
       </c>
       <c r="C8" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F8</f>
-        <v>15750</v>
+        <v>19500</v>
       </c>
       <c r="D8" s="72" t="n">
         <v>12250</v>
       </c>
       <c r="E8" s="71" t="n">
         <f aca="false">C8-D8</f>
-        <v>3500</v>
+        <v>7250</v>
       </c>
       <c r="F8" s="73" t="n">
         <f aca="false">IF(D8=0,"n/a",C8/D8-1)</f>
-        <v>0.285714285714286</v>
+        <v>0.591836734693878</v>
       </c>
       <c r="G8" s="26" t="s">
         <v>182</v>
@@ -3652,18 +3652,18 @@
       </c>
       <c r="C9" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F9</f>
-        <v>8400</v>
+        <v>10500</v>
       </c>
       <c r="D9" s="72" t="n">
         <v>6500</v>
       </c>
       <c r="E9" s="71" t="n">
         <f aca="false">C9-D9</f>
-        <v>1900</v>
+        <v>4000</v>
       </c>
       <c r="F9" s="73" t="n">
         <f aca="false">IF(D9=0,"n/a",C9/D9-1)</f>
-        <v>0.292307692307692</v>
+        <v>0.615384615384615</v>
       </c>
       <c r="G9" s="26" t="s">
         <v>184</v>
@@ -3678,18 +3678,18 @@
       </c>
       <c r="C10" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F10</f>
-        <v>10800</v>
+        <v>13500</v>
       </c>
       <c r="D10" s="72" t="n">
         <v>8500</v>
       </c>
       <c r="E10" s="71" t="n">
         <f aca="false">C10-D10</f>
-        <v>2300</v>
+        <v>5000</v>
       </c>
       <c r="F10" s="73" t="n">
         <f aca="false">IF(D10=0,"n/a",C10/D10-1)</f>
-        <v>0.270588235294118</v>
+        <v>0.588235294117647</v>
       </c>
       <c r="G10" s="26" t="s">
         <v>186</v>
@@ -3704,18 +3704,18 @@
       </c>
       <c r="C11" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F11</f>
-        <v>4100</v>
+        <v>5400</v>
       </c>
       <c r="D11" s="72" t="n">
         <v>3200</v>
       </c>
       <c r="E11" s="71" t="n">
         <f aca="false">C11-D11</f>
-        <v>900</v>
+        <v>2200</v>
       </c>
       <c r="F11" s="73" t="n">
         <f aca="false">IF(D11=0,"n/a",C11/D11-1)</f>
-        <v>0.28125</v>
+        <v>0.6875</v>
       </c>
       <c r="G11" s="26" t="s">
         <v>188</v>
@@ -3730,18 +3730,18 @@
       </c>
       <c r="C12" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F12</f>
-        <v>19900</v>
+        <v>26500</v>
       </c>
       <c r="D12" s="72" t="n">
         <v>15500</v>
       </c>
       <c r="E12" s="71" t="n">
         <f aca="false">C12-D12</f>
-        <v>4400</v>
+        <v>11000</v>
       </c>
       <c r="F12" s="73" t="n">
         <f aca="false">IF(D12=0,"n/a",C12/D12-1)</f>
-        <v>0.283870967741936</v>
+        <v>0.709677419354839</v>
       </c>
       <c r="G12" s="26" t="s">
         <v>190</v>
@@ -3756,18 +3756,18 @@
       </c>
       <c r="C13" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F13</f>
-        <v>26500</v>
+        <v>34500</v>
       </c>
       <c r="D13" s="72" t="n">
         <v>20500</v>
       </c>
       <c r="E13" s="71" t="n">
         <f aca="false">C13-D13</f>
-        <v>6000</v>
+        <v>14000</v>
       </c>
       <c r="F13" s="73" t="n">
         <f aca="false">IF(D13=0,"n/a",C13/D13-1)</f>
-        <v>0.292682926829268</v>
+        <v>0.682926829268293</v>
       </c>
       <c r="G13" s="26" t="s">
         <v>192</v>
@@ -3782,18 +3782,18 @@
       </c>
       <c r="C14" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F14</f>
-        <v>9600</v>
+        <v>12600</v>
       </c>
       <c r="D14" s="72" t="n">
         <v>6300</v>
       </c>
       <c r="E14" s="71" t="n">
         <f aca="false">C14-D14</f>
-        <v>3300</v>
+        <v>6300</v>
       </c>
       <c r="F14" s="73" t="n">
         <f aca="false">IF(D14=0,"n/a",C14/D14-1)</f>
-        <v>0.523809523809524</v>
+        <v>1</v>
       </c>
       <c r="G14" s="26" t="s">
         <v>194</v>
@@ -3808,18 +3808,18 @@
       </c>
       <c r="C15" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F15</f>
-        <v>4500</v>
+        <v>5000</v>
       </c>
       <c r="D15" s="72" t="n">
         <v>2800</v>
       </c>
       <c r="E15" s="71" t="n">
         <f aca="false">C15-D15</f>
-        <v>1700</v>
+        <v>2200</v>
       </c>
       <c r="F15" s="73" t="n">
         <f aca="false">IF(D15=0,"n/a",C15/D15-1)</f>
-        <v>0.607142857142857</v>
+        <v>0.785714285714286</v>
       </c>
       <c r="G15" s="26" t="s">
         <v>196</v>
@@ -3834,18 +3834,18 @@
       </c>
       <c r="C16" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F17</f>
-        <v>4500</v>
+        <v>5500</v>
       </c>
       <c r="D16" s="72" t="n">
         <v>2500</v>
       </c>
       <c r="E16" s="71" t="n">
         <f aca="false">C16-D16</f>
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="F16" s="73" t="n">
         <f aca="false">IF(D16=0,"n/a",C16/D16-1)</f>
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="G16" s="26" t="s">
         <v>198</v>
@@ -3860,18 +3860,18 @@
       </c>
       <c r="C17" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F18</f>
-        <v>8500</v>
+        <v>11500</v>
       </c>
       <c r="D17" s="72" t="n">
         <v>6000</v>
       </c>
       <c r="E17" s="71" t="n">
         <f aca="false">C17-D17</f>
-        <v>2500</v>
+        <v>5500</v>
       </c>
       <c r="F17" s="73" t="n">
         <f aca="false">IF(D17=0,"n/a",C17/D17-1)</f>
-        <v>0.416666666666667</v>
+        <v>0.916666666666667</v>
       </c>
       <c r="G17" s="26" t="s">
         <v>200</v>
@@ -3886,18 +3886,18 @@
       </c>
       <c r="C18" s="71" t="n">
         <f aca="false">'Lot A - Forum'!F19</f>
-        <v>8300</v>
+        <v>9500</v>
       </c>
       <c r="D18" s="72" t="n">
         <v>6500</v>
       </c>
       <c r="E18" s="71" t="n">
         <f aca="false">C18-D18</f>
-        <v>1800</v>
+        <v>3000</v>
       </c>
       <c r="F18" s="73" t="n">
         <f aca="false">IF(D18=0,"n/a",C18/D18-1)</f>
-        <v>0.276923076923077</v>
+        <v>0.461538461538461</v>
       </c>
       <c r="G18" s="26" t="s">
         <v>202</v>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="C25" s="75" t="n">
         <f aca="false">SUM(C5:C24)</f>
-        <v>786030</v>
+        <v>827680</v>
       </c>
       <c r="D25" s="75" t="n">
         <f aca="false">SUM(D5:D24)</f>
@@ -4074,11 +4074,11 @@
       </c>
       <c r="E25" s="75" t="n">
         <f aca="false">C25-D25</f>
-        <v>176525</v>
+        <v>218175</v>
       </c>
       <c r="F25" s="76" t="n">
         <f aca="false">IF(D25=0,"n/a",C25/D25-1)</f>
-        <v>0.289620265625385</v>
+        <v>0.357954405624236</v>
       </c>
       <c r="G25" s="54"/>
     </row>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="C26" s="78" t="n">
         <f aca="false">'Lot A - Forum'!F21+'Lot B - Pavilion'!F12</f>
-        <v>94323.6</v>
+        <v>99321.6</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>